<commit_message>
docs(v23): CHANGE_LOG V23 sprint record + handoff CURRENT STATE (4.05B words, 12.56M sections, headline ~84.9%) + playbook (zero-output breaker idempotent-reseed false-positive + verify-by-id-prefix, CF listing penalty-box → enumerate, inquiries register method) + INQUIRIES_UNIVERSE register + V23 brief archive + corpus status csv/xlsx + seeder checkpoints (S5L enumerated 1-606)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scrutinise-docs/Legislation_Corpus_Status_2026-06-12.xlsx
+++ b/scrutinise-docs/Legislation_Corpus_Status_2026-06-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\scrutinise-prototype\scrutinise-docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD216F46-3B80-4181-84B3-C6707253158D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE4E83D-ED1B-467A-8D5B-494144913905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Corpus Plan" sheetId="1" r:id="rId1"/>
@@ -2202,11 +2202,12 @@
     <col min="5" max="5" width="23.26953125" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="16" width="14" customWidth="1"/>
+    <col min="8" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="34.81640625" customWidth="1"/>
     <col min="17" max="17" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" ht="26" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2259,7 +2260,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -2289,7 +2290,7 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="46" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>18</v>
       </c>
@@ -2334,7 +2335,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
@@ -2379,7 +2380,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>32</v>
       </c>
@@ -2426,7 +2427,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>38</v>
       </c>
@@ -2469,7 +2470,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>41</v>
       </c>
@@ -2514,7 +2515,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>45</v>
       </c>
@@ -2559,7 +2560,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>47</v>
       </c>
@@ -2598,7 +2599,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
@@ -2619,7 +2620,7 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
     </row>
-    <row r="11" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>52</v>
       </c>
@@ -2658,7 +2659,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>56</v>
       </c>
@@ -2705,7 +2706,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>63</v>
       </c>
@@ -2746,7 +2747,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>69</v>
       </c>
@@ -2783,7 +2784,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>77</v>
       </c>
@@ -2804,7 +2805,7 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
     </row>
-    <row r="16" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>78</v>
       </c>
@@ -2845,7 +2846,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>84</v>
       </c>
@@ -2888,7 +2889,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>89</v>
       </c>
@@ -2927,7 +2928,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>93</v>
       </c>
@@ -2966,7 +2967,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>97</v>
       </c>
@@ -3005,7 +3006,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>100</v>
       </c>
@@ -3044,7 +3045,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>107</v>
       </c>
@@ -3081,7 +3082,7 @@
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
     </row>
-    <row r="23" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>111</v>
       </c>
@@ -3124,7 +3125,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>115</v>
       </c>
@@ -3165,7 +3166,7 @@
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
     </row>
-    <row r="25" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>118</v>
       </c>
@@ -3202,7 +3203,7 @@
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
     </row>
-    <row r="26" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>123</v>
       </c>
@@ -3241,7 +3242,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>129</v>
       </c>
@@ -3280,7 +3281,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" s="11" t="s">
         <v>133</v>
       </c>
@@ -3301,7 +3302,7 @@
       <c r="P28" s="11"/>
       <c r="Q28" s="11"/>
     </row>
-    <row r="29" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>134</v>
       </c>
@@ -3346,7 +3347,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>140</v>
       </c>
@@ -3391,7 +3392,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>143</v>
       </c>
@@ -3436,7 +3437,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>148</v>
       </c>
@@ -3479,7 +3480,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>153</v>
       </c>
@@ -3520,7 +3521,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>161</v>
       </c>
@@ -3541,7 +3542,7 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
     </row>
-    <row r="35" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>162</v>
       </c>
@@ -3586,7 +3587,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>169</v>
       </c>
@@ -3631,7 +3632,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>173</v>
       </c>
@@ -3668,7 +3669,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="116.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" ht="46" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>177</v>
       </c>
@@ -3713,7 +3714,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>183</v>
       </c>
@@ -3760,7 +3761,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>189</v>
       </c>
@@ -3807,7 +3808,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>195</v>
       </c>
@@ -3844,7 +3845,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>198</v>
       </c>
@@ -3881,7 +3882,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>202</v>
       </c>
@@ -3918,7 +3919,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>204</v>
       </c>
@@ -3955,7 +3956,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>207</v>
       </c>
@@ -3992,7 +3993,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>211</v>
       </c>
@@ -4029,7 +4030,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>216</v>
       </c>
@@ -4050,7 +4051,7 @@
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
     </row>
-    <row r="48" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>217</v>
       </c>
@@ -4087,7 +4088,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="49" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
         <v>221</v>
       </c>
@@ -4124,7 +4125,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="50" spans="1:17" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>226</v>
       </c>
@@ -4165,7 +4166,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="51" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>232</v>
       </c>
@@ -4186,7 +4187,7 @@
       <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
     </row>
-    <row r="52" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:17" ht="46" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>233</v>
       </c>
@@ -4231,7 +4232,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="53" spans="1:17" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:17" ht="57.5" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
         <v>240</v>
       </c>
@@ -4274,7 +4275,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="54" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>246</v>
       </c>
@@ -4315,7 +4316,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="55" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>250</v>
       </c>
@@ -4356,7 +4357,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="56" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>256</v>
       </c>
@@ -4393,7 +4394,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="57" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>261</v>
       </c>
@@ -4414,7 +4415,7 @@
       <c r="P57" s="2"/>
       <c r="Q57" s="2"/>
     </row>
-    <row r="58" spans="1:17" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>262</v>
       </c>
@@ -4455,7 +4456,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="59" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>268</v>
       </c>
@@ -4500,7 +4501,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="60" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
         <v>274</v>
       </c>
@@ -4543,7 +4544,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="61" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
         <v>280</v>
       </c>
@@ -4580,7 +4581,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="62" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>284</v>
       </c>
@@ -4617,7 +4618,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="63" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>289</v>
       </c>
@@ -4642,7 +4643,7 @@
       <c r="P63" s="4"/>
       <c r="Q63" s="4"/>
     </row>
-    <row r="64" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:17" ht="26" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>290</v>
       </c>
@@ -4663,7 +4664,7 @@
       <c r="P64" s="2"/>
       <c r="Q64" s="2"/>
     </row>
-    <row r="65" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:17" ht="57.5" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
         <v>291</v>
       </c>
@@ -4700,7 +4701,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="66" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:17" ht="46" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>296</v>
       </c>
@@ -4737,7 +4738,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="67" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:17" ht="23" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
         <v>300</v>
       </c>
@@ -4774,7 +4775,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="68" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:17" ht="34.5" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
         <v>304</v>
       </c>
@@ -4811,7 +4812,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="69" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
         <v>308</v>
       </c>
@@ -4848,7 +4849,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="71" spans="1:17" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:17" ht="46" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>310</v>
       </c>

</xml_diff>